<commit_message>
Match web tables to Excel files: show all columns, add Driver Name/Truck to Report
- Fuel table: all 17 columns (A:Q) matching Fuel.xlsx exactly
- Loads table: all 14 columns (A:N) matching Loads.xlsx exactly
- Report Miles table: added Driver Name and Truck columns
- Report Load Summary: all 14 columns matching Loads.xlsx
- Updated Loads/Report CSV exports with all columns
- Updated Add Load modal with all fields (InvoiceID, Load#, Broker, etc.)
- Updated Report parser to handle driverName and truck from Excel
- Regenerated Report.xlsx with Driver Name and Truck columns
- Updated sample data with driverName/truck fields

https://claude.ai/code/session_01UD19NUdXkXWqiRVxgbobqE
</commit_message>
<xml_diff>
--- a/data/Report.xlsx
+++ b/data/Report.xlsx
@@ -397,239 +397,307 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H11"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Driver Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Truck</v>
+      </c>
+      <c r="C1" t="str">
         <v>Date</v>
       </c>
-      <c r="B1" t="str">
+      <c r="D1" t="str">
         <v>Start Odo</v>
       </c>
-      <c r="C1" t="str">
+      <c r="E1" t="str">
         <v>End Odo</v>
       </c>
-      <c r="D1" t="str">
+      <c r="F1" t="str">
         <v>Total Miles</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>Missing Miles</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>Notes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>Driver A</v>
+      </c>
+      <c r="B2" t="str">
+        <v>MPL5046</v>
+      </c>
+      <c r="C2" t="str">
         <v>2025-11-01</v>
       </c>
-      <c r="B2">
+      <c r="D2">
         <v>57685</v>
       </c>
-      <c r="C2">
+      <c r="E2">
         <v>57858</v>
       </c>
-      <c r="D2">
+      <c r="F2">
         <v>173</v>
       </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2" t="str">
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>Driver A</v>
+      </c>
+      <c r="B3" t="str">
+        <v>MPL5046</v>
+      </c>
+      <c r="C3" t="str">
         <v>2025-11-02</v>
       </c>
-      <c r="B3">
+      <c r="D3">
         <v>57858</v>
       </c>
-      <c r="C3">
+      <c r="E3">
         <v>57858</v>
       </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3" t="str">
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>Driver A</v>
+      </c>
+      <c r="B4" t="str">
+        <v>MPL5046</v>
+      </c>
+      <c r="C4" t="str">
         <v>2025-11-03</v>
       </c>
-      <c r="B4">
+      <c r="D4">
         <v>57858</v>
       </c>
-      <c r="C4">
+      <c r="E4">
         <v>57858</v>
       </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
         <v>428</v>
       </c>
-      <c r="F4" t="str">
+      <c r="H4" t="str">
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Driver A</v>
+      </c>
+      <c r="B5" t="str">
+        <v>MPL5046</v>
+      </c>
+      <c r="C5" t="str">
         <v>2025-11-03</v>
       </c>
-      <c r="B5">
+      <c r="D5">
         <v>58286</v>
       </c>
-      <c r="C5">
+      <c r="E5">
         <v>58924</v>
       </c>
-      <c r="D5">
+      <c r="F5">
         <v>638</v>
       </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5" t="str">
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Driver A</v>
+      </c>
+      <c r="B6" t="str">
+        <v>MPL5046</v>
+      </c>
+      <c r="C6" t="str">
         <v>2025-11-04</v>
       </c>
-      <c r="B6">
+      <c r="D6">
         <v>58924</v>
       </c>
-      <c r="C6">
+      <c r="E6">
         <v>59067</v>
       </c>
-      <c r="D6">
+      <c r="F6">
         <v>143</v>
       </c>
-      <c r="E6">
+      <c r="G6">
         <v>136</v>
       </c>
-      <c r="F6" t="str">
+      <c r="H6" t="str">
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>Driver A</v>
+      </c>
+      <c r="B7" t="str">
+        <v>MPL5046</v>
+      </c>
+      <c r="C7" t="str">
         <v>2025-11-04</v>
       </c>
-      <c r="B7">
+      <c r="D7">
         <v>59203</v>
       </c>
-      <c r="C7">
+      <c r="E7">
         <v>59587</v>
       </c>
-      <c r="D7">
+      <c r="F7">
         <v>384</v>
       </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7" t="str">
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>Driver A</v>
+      </c>
+      <c r="B8" t="str">
+        <v>MPL5046</v>
+      </c>
+      <c r="C8" t="str">
         <v>2025-11-05</v>
       </c>
-      <c r="B8">
+      <c r="D8">
         <v>59587</v>
       </c>
-      <c r="C8">
+      <c r="E8">
         <v>60274</v>
       </c>
-      <c r="D8">
+      <c r="F8">
         <v>687</v>
       </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8" t="str">
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="str">
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>Driver A</v>
+      </c>
+      <c r="B9" t="str">
+        <v>MPL5046</v>
+      </c>
+      <c r="C9" t="str">
         <v>2025-11-06</v>
       </c>
-      <c r="B9">
+      <c r="D9">
         <v>60274</v>
       </c>
-      <c r="C9">
+      <c r="E9">
         <v>60274</v>
       </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
         <v>15</v>
       </c>
-      <c r="F9" t="str">
+      <c r="H9" t="str">
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>Driver A</v>
+      </c>
+      <c r="B10" t="str">
+        <v>MPL5046</v>
+      </c>
+      <c r="C10" t="str">
         <v>2025-11-06</v>
       </c>
-      <c r="B10">
+      <c r="D10">
         <v>60289</v>
       </c>
-      <c r="C10">
+      <c r="E10">
         <v>60981</v>
       </c>
-      <c r="D10">
+      <c r="F10">
         <v>692</v>
       </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10" t="str">
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" t="str">
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>Driver A</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MPL5046</v>
+      </c>
+      <c r="C11" t="str">
         <v>2025-11-07</v>
       </c>
-      <c r="B11">
+      <c r="D11">
         <v>60981</v>
       </c>
-      <c r="C11">
+      <c r="E11">
         <v>61048</v>
       </c>
-      <c r="D11">
+      <c r="F11">
         <v>67</v>
       </c>
-      <c r="E11">
+      <c r="G11">
         <v>134</v>
       </c>
-      <c r="F11" t="str">
+      <c r="H11" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>